<commit_message>
ddPCR #13: figuras con SD propia de cada grupo (c- incluido) además de la SD propagada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155wDXPt23zL2HdRwb5YjmM
</commit_message>
<xml_diff>
--- a/analisis/ddpcr_13_resultados.xlsx
+++ b/analisis/ddpcr_13_resultados.xlsx
@@ -351,6 +351,106 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5334000" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5334000" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>117</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5334000" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>117</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5334000" cy="2800350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -2611,7 +2711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2623,6 +2723,8 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2670,10 +2772,20 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>SD propagada (incluye c-)</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del grupo</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del c-</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>ratios_replicas</t>
         </is>
@@ -2708,7 +2820,13 @@
       <c r="H3" t="n">
         <v>0.291</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>0.995;0.748</t>
         </is>
@@ -2743,7 +2861,13 @@
       <c r="H4" t="n">
         <v>0.306</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>1.134;1.154</t>
         </is>
@@ -2778,7 +2902,13 @@
       <c r="H5" t="n">
         <v>0.338</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>0.327</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>0.471;0.008</t>
         </is>
@@ -2813,7 +2943,13 @@
       <c r="H6" t="n">
         <v>0.308</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>0.778;0.483</t>
         </is>
@@ -2864,10 +3000,20 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>SD propagada (incluye c-)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del grupo</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del c-</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>ratios_replicas</t>
         </is>
@@ -2902,7 +3048,13 @@
       <c r="H10" t="n">
         <v>0.291</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>0.995;0.748</t>
         </is>
@@ -2937,7 +3089,13 @@
       <c r="H11" t="n">
         <v>0.306</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>1.134;1.154</t>
         </is>
@@ -2969,7 +3127,10 @@
       <c r="G12" t="n">
         <v>0.471</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>0.471</t>
         </is>
@@ -3004,7 +3165,13 @@
       <c r="H13" t="n">
         <v>0.308</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>0.778;0.483</t>
         </is>
@@ -3055,10 +3222,20 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>SD propagada (incluye c-)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del grupo</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del c-</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>ratios_replicas</t>
         </is>
@@ -3093,7 +3270,13 @@
       <c r="H17" t="n">
         <v>0.217</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>1.044;0.906</t>
         </is>
@@ -3128,7 +3311,13 @@
       <c r="H18" t="n">
         <v>0.25</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>1.222;1.081</t>
         </is>
@@ -3163,7 +3352,13 @@
       <c r="H19" t="n">
         <v>0.366</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>0.523;0.011</t>
         </is>
@@ -3198,7 +3393,13 @@
       <c r="H20" t="n">
         <v>0.258</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>0.747;0.424</t>
         </is>
@@ -3249,10 +3450,20 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>SD propagada (incluye c-)</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del grupo</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>SD propia del c-</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>ratios_replicas</t>
         </is>
@@ -3287,7 +3498,13 @@
       <c r="H24" t="n">
         <v>0.217</v>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>1.044;0.906</t>
         </is>
@@ -3322,7 +3539,13 @@
       <c r="H25" t="n">
         <v>0.25</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>1.222;1.081</t>
         </is>
@@ -3354,7 +3577,10 @@
       <c r="G26" t="n">
         <v>0.523</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>0.523</t>
         </is>
@@ -3389,7 +3615,13 @@
       <c r="H27" t="n">
         <v>0.258</v>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" t="n">
+        <v>0.228</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>0.747;0.424</t>
         </is>
@@ -3406,7 +3638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3420,6 +3652,13 @@
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Medias ± SD por réplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Normalizado vs c- con la SD propia de cada grupo (c- también con su SD)</t>
         </is>
       </c>
     </row>

</xml_diff>